<commit_message>
feat: ScreenQA transfer manifest with auto pair labels from evidence bboxes + base accuracy runner
150 screens / 848 questions / 4056 pairs (T3 3398, T2 100, partial 558) labeled
automatically from answer bounding boxes - replaces 201 manual DocVQA judgments.
Continuous evidence-distance recorded per pair (threshold-free analysis).
IMAGE baseline verified: EM 0.828 / ANLS 0.867 (n=848); 139/150 screens have >=3 correct.

Recommitted after git object corruption from the unclean reboot (11 empty objects
quarantined; history through 6b79933 verified intact).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/experiments/manifests/t4_review.xlsx
+++ b/experiments/manifests/t4_review.xlsx
@@ -2681,7 +2681,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>sqa_val_05331_loc2</t>
+          <t>sqa_val_05332_loc1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2691,24 +2691,24 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>grid3x3</t>
+          <t>half</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>bottom-center</t>
+          <t>top half</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>bottom-center</t>
+          <t>top half</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.5718</v>
+        <v>0.294</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9044</v>
+        <v>0.3518</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -2717,41 +2717,41 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>independent recompute: image W/H read from the actual image file (PIL); center = median over annotator bbox centers from the raw official annotation JSON; label from center fractions (no band filters); seed=44</t>
+          <t>independent recompute: actual image W/H (PIL); median over raw annotator bbox centers; fixed center-to-label rule; seed=44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>sqa_val_06708_loc1</t>
+          <t>sqa_val_07265_loc2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>56219</t>
+          <t>60478</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>half</t>
+          <t>grid3x3</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>top half</t>
+          <t>center</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>top half</t>
+          <t>center</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.1903</v>
+        <v>0.4417</v>
       </c>
       <c r="G3" t="n">
-        <v>0.3706</v>
+        <v>0.5883</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -2760,14 +2760,14 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>independent recompute: image W/H read from the actual image file (PIL); center = median over annotator bbox centers from the raw official annotation JSON; label from center fractions (no band filters); seed=44</t>
+          <t>independent recompute: actual image W/H (PIL); median over raw annotator bbox centers; fixed center-to-label rule; seed=44</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>sqa_val_07265_loc2</t>
+          <t>sqa_val_07266_loc1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2777,24 +2777,24 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>grid3x3</t>
+          <t>half</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>top half</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>center</t>
+          <t>top half</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.4417</v>
+        <v>0.1597</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5883</v>
+        <v>0.268</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -2803,14 +2803,14 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>independent recompute: image W/H read from the actual image file (PIL); center = median over annotator bbox centers from the raw official annotation JSON; label from center fractions (no band filters); seed=44</t>
+          <t>independent recompute: actual image W/H (PIL); median over raw annotator bbox centers; fixed center-to-label rule; seed=44</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>sqa_val_07956_loc2</t>
+          <t>sqa_val_07957_loc1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2820,24 +2820,24 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>grid3x3</t>
+          <t>half</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>middle-left</t>
+          <t>top half</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>middle-left</t>
+          <t>top half</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.2093</v>
+        <v>0.3731</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5263</v>
+        <v>0.1276</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -2846,7 +2846,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>independent recompute: image W/H read from the actual image file (PIL); center = median over annotator bbox centers from the raw official annotation JSON; label from center fractions (no band filters); seed=44</t>
+          <t>independent recompute: actual image W/H (PIL); median over raw annotator bbox centers; fixed center-to-label rule; seed=44</t>
         </is>
       </c>
     </row>
@@ -2889,7 +2889,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>independent recompute: image W/H read from the actual image file (PIL); center = median over annotator bbox centers from the raw official annotation JSON; label from center fractions (no band filters); seed=44</t>
+          <t>independent recompute: actual image W/H (PIL); median over raw annotator bbox centers; fixed center-to-label rule; seed=44</t>
         </is>
       </c>
     </row>
@@ -2932,14 +2932,14 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>independent recompute: image W/H read from the actual image file (PIL); center = median over annotator bbox centers from the raw official annotation JSON; label from center fractions (no band filters); seed=44</t>
+          <t>independent recompute: actual image W/H (PIL); median over raw annotator bbox centers; fixed center-to-label rule; seed=44</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>sqa_val_04721_loc1</t>
+          <t>sqa_val_04725_loc2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2949,24 +2949,24 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>half</t>
+          <t>grid3x3</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>bottom half</t>
+          <t>top-left</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>bottom half</t>
+          <t>top-left</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.3042</v>
+        <v>0.2528</v>
       </c>
       <c r="G8" t="n">
-        <v>0.7651</v>
+        <v>0.2661</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -2975,7 +2975,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>independent recompute: image W/H read from the actual image file (PIL); center = median over annotator bbox centers from the raw official annotation JSON; label from center fractions (no band filters); seed=44</t>
+          <t>independent recompute: actual image W/H (PIL); median over raw annotator bbox centers; fixed center-to-label rule; seed=44</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3018,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>independent recompute: image W/H read from the actual image file (PIL); center = median over annotator bbox centers from the raw official annotation JSON; label from center fractions (no band filters); seed=44</t>
+          <t>independent recompute: actual image W/H (PIL); median over raw annotator bbox centers; fixed center-to-label rule; seed=44</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>independent recompute: image W/H read from the actual image file (PIL); center = median over annotator bbox centers from the raw official annotation JSON; label from center fractions (no band filters); seed=44</t>
+          <t>independent recompute: actual image W/H (PIL); median over raw annotator bbox centers; fixed center-to-label rule; seed=44</t>
         </is>
       </c>
     </row>
@@ -3104,7 +3104,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>independent recompute: image W/H read from the actual image file (PIL); center = median over annotator bbox centers from the raw official annotation JSON; label from center fractions (no band filters); seed=44</t>
+          <t>independent recompute: actual image W/H (PIL); median over raw annotator bbox centers; fixed center-to-label rule; seed=44</t>
         </is>
       </c>
     </row>
@@ -3119,14 +3119,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3141,32 +3135,52 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>image</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>template</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>claimed_answer</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>source_answer_text</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>source_bbox</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>visual_verdict</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>verified_by</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>verified_date</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>note</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>retained_after_audit</t>
         </is>
       </c>
     </row>
@@ -3183,33 +3197,51 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/13920.jpg</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>bottom half</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Recent Search</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>[240, 1732, 408, 1786]</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -3225,33 +3257,51 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/13920.jpg</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>middle-right</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>$41,000</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>[865, 780, 1059, 852]</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -3267,33 +3317,51 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/15084.jpg</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>bottom half</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>24min</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>[871, 1168, 960, 1201]</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>agent+opus_spotcheck</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>에이전트 검증을 Opus가 이미지로 재확인</t>
         </is>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -3309,33 +3377,51 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/15084.jpg</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>middle-right</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>25min</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>[871, 990, 960, 1023]</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -3351,33 +3437,51 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/16339.jpg</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>top half</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>appcrawler6@gmail.com</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>[39, 582, 448, 631]</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -3393,33 +3497,51 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/16339.jpg</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>middle-left</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>883510013034344</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>[39, 1063, 354, 1113]</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -3435,33 +3557,51 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/16692.jpg</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>bottom half</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Sun, Mar 19, 2017 - 4:48 AM</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>[42, 1180, 558, 1237]</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -3477,33 +3617,51 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/16692.jpg</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>middle-left</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>128</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>[128, 1037, 204, 1088]</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -3519,33 +3677,51 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/19288.jpg</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>bottom half</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>9:31 PM CDT</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>[289, 1447, 465, 1488]</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>agent+opus_spotcheck</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
         <is>
           <t>에이전트 검증을 Opus가 이미지로 재확인</t>
         </is>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -3561,33 +3737,51 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/19288.jpg</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>bottom-left</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>March 23, 2017</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>[39, 1447, 251, 1486]</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L11" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -3603,33 +3797,51 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/19964.jpg</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>top half</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>SCRIPTS (30)</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>[427, 248, 652, 297]</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L12" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -3645,33 +3857,51 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/19964.jpg</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>top-center</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>SCRIPTS (30)</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>[427, 248, 652, 297]</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L13" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -3687,33 +3917,51 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/21045.jpg</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>bottom half</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>$ 89.97</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>[574, 1221, 683, 1266]</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L14" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -3729,33 +3977,51 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/21045.jpg</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>middle-right</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Cream and Maroon embr...</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>[561, 1092, 1038, 1154]</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L15" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -3771,33 +4037,51 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/24053.jpg</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>top half</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>appcrawler4@gmail.com</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>[42, 597, 450, 646]</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L16" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -3813,33 +4097,51 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/24053.jpg</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>top-left</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>John Smith</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>[42, 403, 228, 453]</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L17" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -3855,30 +4157,48 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/26974.jpg</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>bottom half</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>0:09</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>[977, 1630, 1079, 1673]</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3893,30 +4213,48 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/26974.jpg</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>top-right</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>0:03</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>[977, 444, 1079, 486]</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3931,33 +4269,51 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/33486.jpg</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>bottom half</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Announce</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>[18, 1335, 218, 1388]</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
         <is>
           <t>'Announce'가 화면에 4회 반복되고 상·하반부에 모두 존재 → 답 모호 (annotation 밖 중복이라 자동 필터가 놓침)</t>
         </is>
+      </c>
+      <c r="L20" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -3973,30 +4329,48 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/33486.jpg</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>top-center</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Champaign, IL</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>[382, 151, 696, 207]</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4011,33 +4385,51 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/34480.jpg</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>top half</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>[787, 351, 950, 416]</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L22" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -4053,33 +4445,51 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/34480.jpg</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>middle-right</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>lbs</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>[876, 740, 956, 803]</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L23" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -4095,30 +4505,48 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/36076.jpg</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>top half</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>SCHEDULE</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>[713, 238, 915, 289]</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4133,30 +4561,48 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/36076.jpg</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>bottom-left</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Android Beam</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>[78, 1672, 254, 1752]</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4171,33 +4617,51 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/38973.jpg</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>bottom half</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>13 May</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>[278, 1450, 379, 1488]</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L26" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -4213,33 +4677,51 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/38973.jpg</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>top-left</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>Edwin &amp; Jhody</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>[42, 470, 504, 552]</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
         <is>
           <t>borderline: 텍스트가 좌/중앙 열에 걸침(중심 규칙으로 left)</t>
         </is>
+      </c>
+      <c r="L27" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -4255,30 +4737,48 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/43764.jpg</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>top half</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>Jun 12, 2015 2:55 PM</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>[174, 658, 461, 693]</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4293,30 +4793,48 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/43764.jpg</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>bottom-center</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>1,883</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>[571, 1716, 666, 1759]</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4331,33 +4849,51 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/53913.jpg</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>top half</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>LIGHTS</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>[338, 96, 475, 139]</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L30" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -4373,33 +4909,51 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/53913.jpg</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>top-left</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>Solid</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>[143, 322, 293, 391]</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L31" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -4415,30 +4969,48 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/54179.jpg</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>top half</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>Gismeteo</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>[373, 155, 787, 247]</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4453,30 +5025,48 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/54179.jpg</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>top-right</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>[704, 462, 1053, 572]</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4491,30 +5081,48 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/56219.jpg</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>top half</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>156</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>[173, 685, 238, 734]</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4529,30 +5137,48 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/56219.jpg</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>bottom-right</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>20 gm</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>[934, 1662, 1038, 1712]</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4567,30 +5193,48 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/60478.jpg</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>top half</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>SOS</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>[137, 495, 208, 534]</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4605,33 +5249,51 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/60478.jpg</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>center</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>appcrawler3@gmail.com</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>[208, 1098, 746, 1161]</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
         <is>
           <t>borderline: 이메일 텍스트가 좌/중앙 열에 걸침(bbox는 텍스트에 밀착)</t>
         </is>
+      </c>
+      <c r="L37" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -4647,30 +5309,48 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/61882.jpg</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>bottom half</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>1:58</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>[269, 1518, 328, 1549]</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4685,30 +5365,48 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/61882.jpg</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>bottom-right</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>1:05</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>[783, 1518, 842, 1551]</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4723,33 +5421,51 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/64175.jpg</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>bottom half</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>10/08</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>[67, 1374, 163, 1423]</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L40" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -4765,33 +5481,51 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/64175.jpg</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>middle-left</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>09/24</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>[67, 1040, 163, 1089]</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L41" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -4807,33 +5541,51 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/64798.jpg</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>bottom half</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>3h</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>[442, 1344, 600, 1407]</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L42" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -4849,33 +5601,51 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/64798.jpg</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>bottom-center</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>mph</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>[442, 1582, 600, 1645]</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L43" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -4891,33 +5661,51 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/66964.jpg</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>bottom half</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>[82, 1322, 232, 1363]</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>agent+opus_spotcheck</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
         <is>
           <t>에이전트 검증을 Opus가 이미지로 재확인</t>
         </is>
+      </c>
+      <c r="L44" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -4933,33 +5721,51 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/66964.jpg</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>top-center</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>modanisa</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>[206, 171, 750, 320]</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>agent+opus_spotcheck</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
         <is>
           <t>에이전트 검증을 Opus가 이미지로 재확인</t>
         </is>
+      </c>
+      <c r="L45" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -4975,33 +5781,51 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/67051.jpg</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>top half</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>Top Stories</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>[252, 189, 554, 301]</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L46" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -5017,33 +5841,51 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/67051.jpg</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>middle-left</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>Iran's Supreme Leader</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>[24, 986, 428, 1037]</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
         <is>
           <t>borderline: 헤드라인 일부 구절의 bbox</t>
         </is>
+      </c>
+      <c r="L47" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -5059,30 +5901,48 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/68259.jpg</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>top half</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>NEWS</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>[369, 194, 711, 299]</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="I48" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5097,30 +5957,48 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/68259.jpg</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>top-center</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>BUNDESLIGA</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>[377, 92, 801, 171]</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5135,33 +6013,51 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/69257.jpg</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>bottom half</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>$38.00</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>[905, 1289, 1038, 1335]</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L50" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -5177,33 +6073,51 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/69257.jpg</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>center</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>$138.37</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>[381, 789, 519, 835]</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="I51" t="inlineStr">
         <is>
           <t>agent+opus_spotcheck</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
         <is>
           <t>에이전트 검증을 Opus가 이미지로 재확인</t>
         </is>
+      </c>
+      <c r="L51" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -5219,33 +6133,51 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/70775.jpg</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
           <t>half</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>top half</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>LOCAL</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>[360, 210, 537, 336]</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>agent</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
         <is>
           <t>에이전트 시각 검증 (표본 5건을 Opus가 재확인해 신뢰성 확인)</t>
         </is>
+      </c>
+      <c r="L52" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -5261,30 +6193,48 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
+          <t>data/screenqa_pilot/70775.jpg</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
           <t>grid3x3</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>top-right</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>16%</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>[974, 462, 1043, 511]</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>opus_direct</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>